<commit_message>
making changes to overall model fit FDRaoQ, CWMs
</commit_message>
<xml_diff>
--- a/df.xlsx
+++ b/df.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stoces\Documents\Cesky_Hradek\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92EC957D-9FBA-4DA3-A119-E4CFEFE56B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2739A767-7EE0-40EF-BD8A-CCE0207FDA3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>